<commit_message>
Zentrale Layout V1.0 finalisierung
</commit_message>
<xml_diff>
--- a/Hardware/SYNCHRO_Booster/BOM_SYNCHRO_Booster.xlsx
+++ b/Hardware/SYNCHRO_Booster/BOM_SYNCHRO_Booster.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jonas\OneDrive - DIG-IT Produktive Umgebung\Desktop\04_BÜP\SYNCHRO\Hardware\SYNCHRO_Booster\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ictedubs-my.sharepoint.com/personal/jonas_henz1_stud_edubs_ch/Documents/Desktop/04_BÜP/SYNCHRO/Hardware/SYNCHRO_Booster/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1306D33-7184-4F96-A0E8-F72974830444}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="6_{A4E94AC5-2DA0-4700-BEFE-0315F7A64D0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EE12FABF-E7B3-4CEF-BE3A-CE7678C9CAAF}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="119">
   <si>
     <t>Projekt:</t>
   </si>
@@ -387,6 +387,9 @@
   </si>
   <si>
     <t>https://www.mouser.ch/en/ProductDetail/Phoenix-Contact/1711738?qs=F79NelsxgYGJoCQSSUE92w%3D%3D</t>
+  </si>
+  <si>
+    <t>Angekommen</t>
   </si>
 </sst>
 </file>
@@ -437,17 +440,27 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4">
     <tableStyle name="Invisible" pivot="0" table="0" count="0" xr9:uid="{8CA2BF20-58F5-4186-8FF3-BFC27E0B33F9}"/>
   </tableStyles>
@@ -784,7 +797,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J51"/>
+  <dimension ref="A1:K35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
@@ -797,7 +810,7 @@
     <col min="8" max="8" width="60.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -817,7 +830,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -837,7 +850,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>12</v>
       </c>
@@ -851,7 +864,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>15</v>
       </c>
@@ -861,29 +874,32 @@
       <c r="C5" t="s">
         <v>97</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" t="s">
+        <v>118</v>
+      </c>
+      <c r="E5" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="F5" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="G5" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="H5" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="H5" t="s">
+      <c r="I5" t="s">
         <v>20</v>
       </c>
-      <c r="I5" t="s">
+      <c r="J5" t="s">
         <v>21</v>
       </c>
-      <c r="J5" t="s">
+      <c r="K5" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>23</v>
       </c>
@@ -894,29 +910,32 @@
         <f>$B$3*B6</f>
         <v>30</v>
       </c>
-      <c r="D6" s="1">
+      <c r="D6" t="s">
+        <v>98</v>
+      </c>
+      <c r="E6" s="1">
         <v>40</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="G6" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="H6" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="H6" t="s">
-        <v>28</v>
       </c>
       <c r="I6" t="s">
         <v>28</v>
       </c>
       <c r="J6" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+        <v>28</v>
+      </c>
+      <c r="K6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>29</v>
       </c>
@@ -927,29 +946,32 @@
         <f t="shared" ref="C7:C16" si="0">$B$3*B7</f>
         <v>12</v>
       </c>
-      <c r="D7" s="1">
+      <c r="D7" t="s">
+        <v>98</v>
+      </c>
+      <c r="E7" s="1">
         <v>15</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="F7" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="G7" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="H7" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="H7" t="s">
-        <v>32</v>
       </c>
       <c r="I7" t="s">
         <v>32</v>
       </c>
       <c r="J7" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+        <v>32</v>
+      </c>
+      <c r="K7" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>33</v>
       </c>
@@ -960,29 +982,32 @@
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8" t="s">
+        <v>98</v>
+      </c>
+      <c r="E8" s="1">
         <v>10</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="F8" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="G8" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="H8" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="H8" t="s">
-        <v>28</v>
       </c>
       <c r="I8" t="s">
         <v>28</v>
       </c>
       <c r="J8" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+        <v>28</v>
+      </c>
+      <c r="K8" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>36</v>
       </c>
@@ -993,29 +1018,32 @@
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="D9" s="1">
+      <c r="D9" t="s">
+        <v>98</v>
+      </c>
+      <c r="E9" s="1">
         <v>20</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="F9" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="G9" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="H9" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="H9" t="s">
-        <v>39</v>
       </c>
       <c r="I9" t="s">
         <v>39</v>
       </c>
       <c r="J9" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+        <v>39</v>
+      </c>
+      <c r="K9" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>40</v>
       </c>
@@ -1026,29 +1054,32 @@
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="D10" s="1">
+      <c r="D10" t="s">
+        <v>98</v>
+      </c>
+      <c r="E10" s="1">
         <v>10</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="F10" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="G10" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="G10" s="1" t="s">
+      <c r="H10" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="H10" t="s">
-        <v>39</v>
       </c>
       <c r="I10" t="s">
         <v>39</v>
       </c>
       <c r="J10" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+        <v>39</v>
+      </c>
+      <c r="K10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>42</v>
       </c>
@@ -1059,29 +1090,32 @@
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="D11" s="1">
+      <c r="D11" t="s">
+        <v>98</v>
+      </c>
+      <c r="E11" s="1">
         <v>20</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="F11" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="G11" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="G11" s="1" t="s">
+      <c r="H11" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="H11" t="s">
-        <v>44</v>
       </c>
       <c r="I11" t="s">
         <v>44</v>
       </c>
       <c r="J11" t="s">
+        <v>44</v>
+      </c>
+      <c r="K11" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>46</v>
       </c>
@@ -1092,29 +1126,32 @@
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="D12" s="1">
+      <c r="D12" t="s">
+        <v>98</v>
+      </c>
+      <c r="E12" s="1">
         <v>10</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="F12" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="G12" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="G12" s="1" t="s">
+      <c r="H12" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="H12" t="s">
-        <v>48</v>
       </c>
       <c r="I12" t="s">
         <v>48</v>
       </c>
       <c r="J12" t="s">
+        <v>48</v>
+      </c>
+      <c r="K12" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>50</v>
       </c>
@@ -1125,26 +1162,26 @@
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="D13" t="s">
-        <v>98</v>
-      </c>
       <c r="E13" t="s">
+        <v>98</v>
+      </c>
+      <c r="F13" t="s">
         <v>51</v>
       </c>
-      <c r="G13" t="s">
-        <v>25</v>
-      </c>
       <c r="H13" t="s">
-        <v>52</v>
+        <v>25</v>
       </c>
       <c r="I13" t="s">
         <v>52</v>
       </c>
       <c r="J13" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+        <v>52</v>
+      </c>
+      <c r="K13" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>53</v>
       </c>
@@ -1155,29 +1192,32 @@
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="D14" s="1">
+      <c r="D14" t="s">
+        <v>98</v>
+      </c>
+      <c r="E14" s="1">
         <v>10</v>
       </c>
-      <c r="E14" s="1" t="s">
+      <c r="F14" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="F14" s="2" t="s">
+      <c r="G14" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="G14" s="1" t="s">
+      <c r="H14" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="H14" t="s">
-        <v>55</v>
       </c>
       <c r="I14" t="s">
         <v>55</v>
       </c>
       <c r="J14" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+        <v>55</v>
+      </c>
+      <c r="K14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>56</v>
       </c>
@@ -1188,29 +1228,32 @@
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="D15" s="1">
-        <v>6</v>
-      </c>
-      <c r="E15" s="1" t="s">
+      <c r="D15" t="s">
+        <v>98</v>
+      </c>
+      <c r="E15" s="1">
+        <v>6</v>
+      </c>
+      <c r="F15" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="F15" s="2" t="s">
+      <c r="G15" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="G15" s="1" t="s">
+      <c r="H15" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="H15" t="s">
-        <v>58</v>
       </c>
       <c r="I15" t="s">
         <v>58</v>
       </c>
       <c r="J15" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+        <v>58</v>
+      </c>
+      <c r="K15" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>113</v>
       </c>
@@ -1221,29 +1264,32 @@
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="D16" s="1">
+      <c r="D16" t="s">
+        <v>98</v>
+      </c>
+      <c r="E16" s="1">
         <v>12</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="F16" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="F16" s="2" t="s">
+      <c r="G16" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="G16" s="1" t="s">
+      <c r="H16" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="H16" t="s">
-        <v>60</v>
       </c>
       <c r="I16" t="s">
         <v>60</v>
       </c>
       <c r="J16" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+        <v>60</v>
+      </c>
+      <c r="K16" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>61</v>
       </c>
@@ -1254,29 +1300,32 @@
         <f t="shared" ref="C17:C31" si="1">$B$3*B17</f>
         <v>6</v>
       </c>
-      <c r="D17" s="1">
+      <c r="D17" t="s">
+        <v>98</v>
+      </c>
+      <c r="E17" s="1">
         <v>20</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="F17" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="F17" s="2" t="s">
+      <c r="G17" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="G17" s="1" t="s">
+      <c r="H17" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="H17" t="s">
-        <v>63</v>
       </c>
       <c r="I17" t="s">
         <v>63</v>
       </c>
       <c r="J17" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+        <v>63</v>
+      </c>
+      <c r="K17" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>64</v>
       </c>
@@ -1287,26 +1336,26 @@
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="D18" t="s">
-        <v>98</v>
-      </c>
       <c r="E18" t="s">
+        <v>98</v>
+      </c>
+      <c r="F18" t="s">
         <v>51</v>
       </c>
-      <c r="G18" t="s">
-        <v>25</v>
-      </c>
       <c r="H18" t="s">
-        <v>65</v>
+        <v>25</v>
       </c>
       <c r="I18" t="s">
         <v>65</v>
       </c>
       <c r="J18" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+        <v>65</v>
+      </c>
+      <c r="K18" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>66</v>
       </c>
@@ -1317,29 +1366,32 @@
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="D19" s="1">
+      <c r="D19" t="s">
+        <v>98</v>
+      </c>
+      <c r="E19" s="1">
         <v>8</v>
       </c>
-      <c r="E19" s="1" t="s">
+      <c r="F19" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="F19" s="2" t="s">
+      <c r="G19" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="G19" s="1" t="s">
+      <c r="H19" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="H19" t="s">
-        <v>68</v>
       </c>
       <c r="I19" t="s">
         <v>68</v>
       </c>
       <c r="J19" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+        <v>68</v>
+      </c>
+      <c r="K19" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>69</v>
       </c>
@@ -1350,29 +1402,32 @@
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="D20" s="1">
+      <c r="D20" t="s">
+        <v>98</v>
+      </c>
+      <c r="E20" s="1">
         <v>10</v>
       </c>
-      <c r="E20" s="1" t="s">
+      <c r="F20" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="F20" s="2" t="s">
+      <c r="G20" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="G20" s="1" t="s">
+      <c r="H20" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="H20" t="s">
-        <v>71</v>
       </c>
       <c r="I20" t="s">
         <v>71</v>
       </c>
       <c r="J20" t="s">
+        <v>71</v>
+      </c>
+      <c r="K20" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>73</v>
       </c>
@@ -1383,26 +1438,26 @@
         <f t="shared" si="1"/>
         <v>24</v>
       </c>
-      <c r="D21" t="s">
-        <v>98</v>
-      </c>
       <c r="E21" t="s">
+        <v>98</v>
+      </c>
+      <c r="F21" t="s">
         <v>51</v>
       </c>
-      <c r="G21" t="s">
-        <v>25</v>
-      </c>
       <c r="H21" t="s">
-        <v>75</v>
+        <v>25</v>
       </c>
       <c r="I21" t="s">
         <v>75</v>
       </c>
       <c r="J21" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+        <v>75</v>
+      </c>
+      <c r="K21" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>76</v>
       </c>
@@ -1413,26 +1468,26 @@
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="D22" t="s">
-        <v>98</v>
-      </c>
       <c r="E22" t="s">
+        <v>98</v>
+      </c>
+      <c r="F22" t="s">
         <v>51</v>
       </c>
-      <c r="G22" t="s">
-        <v>25</v>
-      </c>
       <c r="H22" t="s">
-        <v>75</v>
+        <v>25</v>
       </c>
       <c r="I22" t="s">
         <v>75</v>
       </c>
       <c r="J22" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+        <v>75</v>
+      </c>
+      <c r="K22" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>77</v>
       </c>
@@ -1443,26 +1498,26 @@
         <f t="shared" si="1"/>
         <v>18</v>
       </c>
-      <c r="D23" t="s">
-        <v>98</v>
-      </c>
       <c r="E23" t="s">
+        <v>98</v>
+      </c>
+      <c r="F23" t="s">
         <v>51</v>
       </c>
-      <c r="G23" t="s">
-        <v>25</v>
-      </c>
       <c r="H23" t="s">
-        <v>75</v>
+        <v>25</v>
       </c>
       <c r="I23" t="s">
         <v>75</v>
       </c>
       <c r="J23" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+        <v>75</v>
+      </c>
+      <c r="K23" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>78</v>
       </c>
@@ -1473,26 +1528,26 @@
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="D24" t="s">
-        <v>98</v>
-      </c>
       <c r="E24" t="s">
+        <v>98</v>
+      </c>
+      <c r="F24" t="s">
         <v>51</v>
       </c>
-      <c r="G24" t="s">
-        <v>25</v>
-      </c>
       <c r="H24" t="s">
-        <v>75</v>
+        <v>25</v>
       </c>
       <c r="I24" t="s">
         <v>75</v>
       </c>
       <c r="J24" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+        <v>75</v>
+      </c>
+      <c r="K24" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>79</v>
       </c>
@@ -1503,26 +1558,26 @@
         <f t="shared" si="1"/>
         <v>12</v>
       </c>
-      <c r="D25" t="s">
-        <v>98</v>
-      </c>
       <c r="E25" t="s">
+        <v>98</v>
+      </c>
+      <c r="F25" t="s">
         <v>51</v>
       </c>
-      <c r="G25" t="s">
-        <v>25</v>
-      </c>
       <c r="H25" t="s">
-        <v>75</v>
+        <v>25</v>
       </c>
       <c r="I25" t="s">
         <v>75</v>
       </c>
       <c r="J25" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+        <v>75</v>
+      </c>
+      <c r="K25" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>80</v>
       </c>
@@ -1533,26 +1588,26 @@
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="D26" t="s">
-        <v>98</v>
-      </c>
       <c r="E26" t="s">
+        <v>98</v>
+      </c>
+      <c r="F26" t="s">
         <v>51</v>
       </c>
-      <c r="G26" t="s">
-        <v>25</v>
-      </c>
       <c r="H26" t="s">
-        <v>75</v>
+        <v>25</v>
       </c>
       <c r="I26" t="s">
         <v>75</v>
       </c>
       <c r="J26" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+        <v>75</v>
+      </c>
+      <c r="K26" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>81</v>
       </c>
@@ -1563,26 +1618,26 @@
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="D27" t="s">
-        <v>98</v>
-      </c>
       <c r="E27" t="s">
+        <v>98</v>
+      </c>
+      <c r="F27" t="s">
         <v>51</v>
       </c>
-      <c r="G27" t="s">
-        <v>25</v>
-      </c>
       <c r="H27" t="s">
-        <v>82</v>
+        <v>25</v>
       </c>
       <c r="I27" t="s">
         <v>82</v>
       </c>
       <c r="J27" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+        <v>82</v>
+      </c>
+      <c r="K27" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>83</v>
       </c>
@@ -1593,29 +1648,32 @@
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="D28" s="1">
-        <v>6</v>
-      </c>
-      <c r="E28" s="1" t="s">
+      <c r="D28" t="s">
+        <v>98</v>
+      </c>
+      <c r="E28" s="1">
+        <v>6</v>
+      </c>
+      <c r="F28" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="F28" s="2" t="s">
+      <c r="G28" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="G28" s="1" t="s">
+      <c r="H28" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="H28" t="s">
-        <v>85</v>
       </c>
       <c r="I28" t="s">
         <v>85</v>
       </c>
       <c r="J28" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
+        <v>85</v>
+      </c>
+      <c r="K28" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>86</v>
       </c>
@@ -1626,29 +1684,32 @@
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="D29" s="1">
+      <c r="D29" t="s">
+        <v>98</v>
+      </c>
+      <c r="E29" s="1">
         <v>10</v>
       </c>
-      <c r="E29" s="1" t="s">
+      <c r="F29" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="F29" s="2" t="s">
+      <c r="G29" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="G29" s="1" t="s">
+      <c r="H29" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="H29" t="s">
-        <v>88</v>
       </c>
       <c r="I29" t="s">
         <v>88</v>
       </c>
       <c r="J29" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+        <v>88</v>
+      </c>
+      <c r="K29" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>89</v>
       </c>
@@ -1659,29 +1720,32 @@
         <f t="shared" si="1"/>
         <v>12</v>
       </c>
-      <c r="D30" s="1">
+      <c r="D30" t="s">
+        <v>98</v>
+      </c>
+      <c r="E30" s="1">
         <v>20</v>
       </c>
-      <c r="E30" s="1" t="s">
+      <c r="F30" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="F30" s="2" t="s">
+      <c r="G30" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="G30" s="1" t="s">
+      <c r="H30" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="H30" t="s">
-        <v>88</v>
       </c>
       <c r="I30" t="s">
         <v>88</v>
       </c>
       <c r="J30" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+        <v>88</v>
+      </c>
+      <c r="K30" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>91</v>
       </c>
@@ -1692,31 +1756,32 @@
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="D31" s="1">
+      <c r="D31" t="s">
+        <v>98</v>
+      </c>
+      <c r="E31" s="1">
         <v>10</v>
       </c>
-      <c r="E31" s="1" t="s">
+      <c r="F31" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="F31" s="2" t="s">
+      <c r="G31" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="G31" s="1" t="s">
+      <c r="H31" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="H31" t="s">
-        <v>93</v>
       </c>
       <c r="I31" t="s">
         <v>93</v>
       </c>
       <c r="J31" t="s">
+        <v>93</v>
+      </c>
+      <c r="K31" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="34" spans="4:8" x14ac:dyDescent="0.35">
-      <c r="D34" s="3"/>
-      <c r="E34" s="3"/>
+    <row r="34" spans="7:8" x14ac:dyDescent="0.35">
       <c r="G34" t="s">
         <v>95</v>
       </c>
@@ -1724,9 +1789,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="4:8" x14ac:dyDescent="0.35">
-      <c r="D35" s="3"/>
-      <c r="E35" s="3"/>
+    <row r="35" spans="7:8" x14ac:dyDescent="0.35">
       <c r="G35" t="s">
         <v>96</v>
       </c>
@@ -1734,89 +1797,30 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="4:8" x14ac:dyDescent="0.35">
-      <c r="D36" s="3"/>
-      <c r="E36" s="3"/>
-    </row>
-    <row r="37" spans="4:8" x14ac:dyDescent="0.35">
-      <c r="D37" s="3"/>
-      <c r="E37" s="3"/>
-    </row>
-    <row r="38" spans="4:8" x14ac:dyDescent="0.35">
-      <c r="D38" s="3"/>
-      <c r="E38" s="3"/>
-    </row>
-    <row r="39" spans="4:8" x14ac:dyDescent="0.35">
-      <c r="D39" s="3"/>
-      <c r="E39" s="3"/>
-    </row>
-    <row r="40" spans="4:8" x14ac:dyDescent="0.35">
-      <c r="D40" s="3"/>
-      <c r="E40" s="3"/>
-    </row>
-    <row r="41" spans="4:8" x14ac:dyDescent="0.35">
-      <c r="D41" s="3"/>
-      <c r="E41" s="3"/>
-    </row>
-    <row r="42" spans="4:8" x14ac:dyDescent="0.35">
-      <c r="D42" s="3"/>
-      <c r="E42" s="3"/>
-    </row>
-    <row r="43" spans="4:8" x14ac:dyDescent="0.35">
-      <c r="D43" s="3"/>
-      <c r="E43" s="3"/>
-    </row>
-    <row r="44" spans="4:8" x14ac:dyDescent="0.35">
-      <c r="D44" s="3"/>
-      <c r="E44" s="3"/>
-    </row>
-    <row r="45" spans="4:8" x14ac:dyDescent="0.35">
-      <c r="D45" s="3"/>
-      <c r="E45" s="3"/>
-    </row>
-    <row r="46" spans="4:8" x14ac:dyDescent="0.35">
-      <c r="D46" s="3"/>
-      <c r="E46" s="3"/>
-    </row>
-    <row r="47" spans="4:8" x14ac:dyDescent="0.35">
-      <c r="D47" s="3"/>
-      <c r="E47" s="3"/>
-    </row>
-    <row r="48" spans="4:8" x14ac:dyDescent="0.35">
-      <c r="D48" s="3"/>
-      <c r="E48" s="3"/>
-    </row>
-    <row r="49" spans="4:5" x14ac:dyDescent="0.35">
-      <c r="D49" s="3"/>
-      <c r="E49" s="3"/>
-    </row>
-    <row r="50" spans="4:5" x14ac:dyDescent="0.35">
-      <c r="D50" s="3"/>
-      <c r="E50" s="3"/>
-    </row>
-    <row r="51" spans="4:5" x14ac:dyDescent="0.35">
-      <c r="D51" s="3"/>
-      <c r="E51" s="3"/>
-    </row>
   </sheetData>
+  <conditionalFormatting sqref="D6:D31">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
+      <formula>"x"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="F29" r:id="rId1" xr:uid="{0A8DAB46-FB9B-4F7B-A55E-B7FCFAD51833}"/>
-    <hyperlink ref="F30" r:id="rId2" xr:uid="{0980E79F-FBF3-42BB-9DE0-BE508B2D0D68}"/>
-    <hyperlink ref="F31" r:id="rId3" xr:uid="{D1690A06-7338-4AEF-A65E-7F1683906339}"/>
-    <hyperlink ref="F6" r:id="rId4" xr:uid="{81A50C11-649E-439F-81F3-C1FF31814EC5}"/>
-    <hyperlink ref="F7" r:id="rId5" xr:uid="{6F9511FF-E870-4E0A-8D34-3F3AA047A04B}"/>
-    <hyperlink ref="F8" r:id="rId6" xr:uid="{5989DEFD-C839-470E-95A7-9E51C0091C03}"/>
-    <hyperlink ref="F9" r:id="rId7" xr:uid="{07EAA88D-ED39-48AA-BFC8-2346E7635374}"/>
-    <hyperlink ref="F10" r:id="rId8" xr:uid="{925B90A7-F5C1-42F1-90AA-937DAF19DD64}"/>
-    <hyperlink ref="F11" r:id="rId9" xr:uid="{D4D5C0BE-0156-415F-84DF-FF38F66BE6AE}"/>
-    <hyperlink ref="F12" r:id="rId10" xr:uid="{98163EB9-9FD8-4BB8-8DA7-A9A076C528B6}"/>
-    <hyperlink ref="F14" r:id="rId11" xr:uid="{F62C3FDB-8593-4540-ABD6-49F26A3AF0A0}"/>
-    <hyperlink ref="F15" r:id="rId12" xr:uid="{84DCA40F-7B7B-40EB-87E8-ABF759DAEBDC}"/>
-    <hyperlink ref="F16" r:id="rId13" xr:uid="{BD827227-6A6A-4898-802F-7098A8B54660}"/>
-    <hyperlink ref="F17" r:id="rId14" xr:uid="{5EBE495F-17AB-4142-AAE9-3109BE74CE0C}"/>
-    <hyperlink ref="F19" r:id="rId15" xr:uid="{54B3042E-16AA-4EA7-B7E1-FF679E633297}"/>
-    <hyperlink ref="F20" r:id="rId16" xr:uid="{829CE8B6-6526-44C6-907C-CF0EFB03F9C0}"/>
-    <hyperlink ref="F28" r:id="rId17" xr:uid="{60E1A3ED-09AA-4DCE-A604-94A25059BA44}"/>
+    <hyperlink ref="G29" r:id="rId1" xr:uid="{0A8DAB46-FB9B-4F7B-A55E-B7FCFAD51833}"/>
+    <hyperlink ref="G30" r:id="rId2" xr:uid="{0980E79F-FBF3-42BB-9DE0-BE508B2D0D68}"/>
+    <hyperlink ref="G31" r:id="rId3" xr:uid="{D1690A06-7338-4AEF-A65E-7F1683906339}"/>
+    <hyperlink ref="G6" r:id="rId4" xr:uid="{81A50C11-649E-439F-81F3-C1FF31814EC5}"/>
+    <hyperlink ref="G7" r:id="rId5" xr:uid="{6F9511FF-E870-4E0A-8D34-3F3AA047A04B}"/>
+    <hyperlink ref="G8" r:id="rId6" xr:uid="{5989DEFD-C839-470E-95A7-9E51C0091C03}"/>
+    <hyperlink ref="G9" r:id="rId7" xr:uid="{07EAA88D-ED39-48AA-BFC8-2346E7635374}"/>
+    <hyperlink ref="G10" r:id="rId8" xr:uid="{925B90A7-F5C1-42F1-90AA-937DAF19DD64}"/>
+    <hyperlink ref="G11" r:id="rId9" xr:uid="{D4D5C0BE-0156-415F-84DF-FF38F66BE6AE}"/>
+    <hyperlink ref="G12" r:id="rId10" xr:uid="{98163EB9-9FD8-4BB8-8DA7-A9A076C528B6}"/>
+    <hyperlink ref="G14" r:id="rId11" xr:uid="{F62C3FDB-8593-4540-ABD6-49F26A3AF0A0}"/>
+    <hyperlink ref="G15" r:id="rId12" xr:uid="{84DCA40F-7B7B-40EB-87E8-ABF759DAEBDC}"/>
+    <hyperlink ref="G16" r:id="rId13" xr:uid="{BD827227-6A6A-4898-802F-7098A8B54660}"/>
+    <hyperlink ref="G17" r:id="rId14" xr:uid="{5EBE495F-17AB-4142-AAE9-3109BE74CE0C}"/>
+    <hyperlink ref="G19" r:id="rId15" xr:uid="{54B3042E-16AA-4EA7-B7E1-FF679E633297}"/>
+    <hyperlink ref="G20" r:id="rId16" xr:uid="{829CE8B6-6526-44C6-907C-CF0EFB03F9C0}"/>
+    <hyperlink ref="G28" r:id="rId17" xr:uid="{60E1A3ED-09AA-4DCE-A604-94A25059BA44}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <ignoredErrors>

</xml_diff>